<commit_message>
Planilha modelo: listas suspensas sem linhas vazias
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0183SZjsW45vA4LqbeF8Lqx2
</commit_message>
<xml_diff>
--- a/modelo/Diario_de_Trades.xlsx
+++ b/modelo/Diario_de_Trades.xlsx
@@ -15887,13 +15887,13 @@
       <formula1>"Compra,Venda"</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I1001" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Setups!$A$2:$A$100</formula1>
+      <formula1>OFFSET(Setups!$A$2,0,0,MAX(1,COUNTA(Setups!$A$2:$A$500)),1)</formula1>
     </dataValidation>
     <dataValidation sqref="J2:J1001" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Setups!$D$2:$D$50</formula1>
+      <formula1>OFFSET(Setups!$D$2,0,0,MAX(1,COUNTA(Setups!$D$2:$D$500)),1)</formula1>
     </dataValidation>
     <dataValidation sqref="K2:K1001" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Setups!$E$2:$E$50</formula1>
+      <formula1>OFFSET(Setups!$E$2,0,0,MAX(1,COUNTA(Setups!$E$2:$E$500)),1)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -31041,13 +31041,13 @@
       <formula1>"Compra,Venda"</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I1001" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Setups!$A$2:$A$100</formula1>
+      <formula1>OFFSET(Setups!$A$2,0,0,MAX(1,COUNTA(Setups!$A$2:$A$500)),1)</formula1>
     </dataValidation>
     <dataValidation sqref="J2:J1001" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Setups!$D$2:$D$50</formula1>
+      <formula1>OFFSET(Setups!$D$2,0,0,MAX(1,COUNTA(Setups!$D$2:$D$500)),1)</formula1>
     </dataValidation>
     <dataValidation sqref="K2:K1001" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Setups!$E$2:$E$50</formula1>
+      <formula1>OFFSET(Setups!$E$2,0,0,MAX(1,COUNTA(Setups!$E$2:$E$500)),1)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -46194,13 +46194,13 @@
       <formula1>"Compra,Venda"</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I1001" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Setups!$A$2:$A$100</formula1>
+      <formula1>OFFSET(Setups!$A$2,0,0,MAX(1,COUNTA(Setups!$A$2:$A$500)),1)</formula1>
     </dataValidation>
     <dataValidation sqref="J2:J1001" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Setups!$D$2:$D$50</formula1>
+      <formula1>OFFSET(Setups!$D$2,0,0,MAX(1,COUNTA(Setups!$D$2:$D$500)),1)</formula1>
     </dataValidation>
     <dataValidation sqref="K2:K1001" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Setups!$E$2:$E$50</formula1>
+      <formula1>OFFSET(Setups!$E$2,0,0,MAX(1,COUNTA(Setups!$E$2:$E$500)),1)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>